<commit_message>
update sheet for new tests
</commit_message>
<xml_diff>
--- a/d.BOBO Handoffs.xlsx
+++ b/d.BOBO Handoffs.xlsx
@@ -5,6 +5,8 @@
   <sheets>
     <sheet state="visible" name="d.BOBO Handoffs" sheetId="1" r:id="rId5"/>
     <sheet state="visible" name="d.BOBO Custom" sheetId="2" r:id="rId6"/>
+    <sheet state="visible" name="d.BOBO SIPOC" sheetId="3" r:id="rId7"/>
+    <sheet state="visible" name="d.BOBO Funnel" sheetId="4" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr/>
@@ -12,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="136" uniqueCount="61">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="188" uniqueCount="92">
   <si>
     <t>Timestamp</t>
   </si>
@@ -176,13 +178,15 @@
     <t>In 1 year, we are a reliable testing framework with a reputation for accuracy and speed.</t>
   </si>
   <si>
-    <t>Customer Profile</t>
+    <t>Customer 
+Profile</t>
   </si>
   <si>
     <t>Needs Answers</t>
   </si>
   <si>
-    <t>Custom Statement</t>
+    <t>Custom 
+Statement</t>
   </si>
   <si>
     <t>This is a test profile.</t>
@@ -195,6 +199,103 @@
   </si>
   <si>
     <t>3-SIPOC</t>
+  </si>
+  <si>
+    <t>Suppliers</t>
+  </si>
+  <si>
+    <t>Inputs</t>
+  </si>
+  <si>
+    <t>Process Steps</t>
+  </si>
+  <si>
+    <t>Outputs</t>
+  </si>
+  <si>
+    <t>Customers</t>
+  </si>
+  <si>
+    <t>Shop</t>
+  </si>
+  <si>
+    <t>COQ Snapshot</t>
+  </si>
+  <si>
+    <t>test suppliers</t>
+  </si>
+  <si>
+    <t>test inputs</t>
+  </si>
+  <si>
+    <t>test steps</t>
+  </si>
+  <si>
+    <t>test outputs</t>
+  </si>
+  <si>
+    <t>test customers</t>
+  </si>
+  <si>
+    <t>test shop</t>
+  </si>
+  <si>
+    <t>test number</t>
+  </si>
+  <si>
+    <t>4-funnel</t>
+  </si>
+  <si>
+    <t>Starting 
+Customer</t>
+  </si>
+  <si>
+    <t>Awareness 
+Channels</t>
+  </si>
+  <si>
+    <t>Consideration 
+Assets</t>
+  </si>
+  <si>
+    <t>Sale Process</t>
+  </si>
+  <si>
+    <t>Account Mgmt</t>
+  </si>
+  <si>
+    <t>Brand Words</t>
+  </si>
+  <si>
+    <t>Launch 
+Readiness</t>
+  </si>
+  <si>
+    <t>48hr Action</t>
+  </si>
+  <si>
+    <t>test customer</t>
+  </si>
+  <si>
+    <t>test channels</t>
+  </si>
+  <si>
+    <t>test assets</t>
+  </si>
+  <si>
+    <t>test sale process</t>
+  </si>
+  <si>
+    <t>test acct mgmt</t>
+  </si>
+  <si>
+    <t>test words</t>
+  </si>
+  <si>
+    <t>test readiness</t>
+  </si>
+  <si>
+    <t>test action</t>
   </si>
 </sst>
 </file>
@@ -269,6 +370,14 @@
 </file>
 
 <file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
+</file>
+
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
+</file>
+
+<file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
 </file>
 
@@ -935,6 +1044,9 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
   <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <cols>
+    <col customWidth="1" min="5" max="5" width="17.75"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
@@ -967,7 +1079,7 @@
     </row>
     <row r="2">
       <c r="A2" s="2">
-        <v>46138.901088541665</v>
+        <v>46141.97176835648</v>
       </c>
       <c r="B2" s="3" t="s">
         <v>22</v>
@@ -992,6 +1104,200 @@
       </c>
       <c r="I2" s="3" t="s">
         <v>60</v>
+      </c>
+    </row>
+  </sheetData>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="0" summaryRight="0"/>
+  </sheetPr>
+  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2">
+        <v>46141.97639885417</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="G2" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="H2" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="I2" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="J2" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="K2" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="L2" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="M2" s="3" t="s">
+        <v>75</v>
+      </c>
+    </row>
+  </sheetData>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="0" summaryRight="0"/>
+  </sheetPr>
+  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2">
+        <v>46141.97661395834</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="G2" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="H2" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="I2" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="J2" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="K2" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="L2" s="3" t="s">
+        <v>91</v>
+      </c>
+      <c r="M2" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="N2" s="3" t="s">
+        <v>21</v>
       </c>
     </row>
   </sheetData>

</xml_diff>